<commit_message>
Add journal excel file
</commit_message>
<xml_diff>
--- a/journals/journal-2026-03-29.xlsx
+++ b/journals/journal-2026-03-29.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -423,27 +423,67 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>building this/trouble shooting</v>
+        <v>Learn</v>
       </c>
       <c r="B2" t="str">
         <v>Learning</v>
       </c>
       <c r="C2" t="str">
-        <v>09:01</v>
+        <v>10:35</v>
       </c>
       <c r="D2" t="str">
-        <v>09:36</v>
+        <v>10:54</v>
       </c>
       <c r="E2">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="F2" t="str">
-        <v>more like building ts</v>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Nail cut</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Necessity</v>
+      </c>
+      <c r="C3" t="str">
+        <v>10:54</v>
+      </c>
+      <c r="D3" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="E3">
+        <v>11</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>AWS AI pract</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Learning</v>
+      </c>
+      <c r="C4" t="str">
+        <v>11:05</v>
+      </c>
+      <c r="D4" t="str">
+        <v>12:27</v>
+      </c>
+      <c r="E4">
+        <v>82</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -465,7 +505,7 @@
         <v>Entry Count</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -473,7 +513,7 @@
         <v>Total Minutes</v>
       </c>
       <c r="B3">
-        <v>35</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
@@ -481,7 +521,7 @@
         <v>Total Hours</v>
       </c>
       <c r="B4" t="str">
-        <v>0.58</v>
+        <v>1.87</v>
       </c>
     </row>
   </sheetData>
@@ -508,7 +548,7 @@
         <v>Generated</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-03-29T16:39:16.462Z</v>
+        <v>2026-03-29T19:27:37.976Z</v>
       </c>
     </row>
     <row r="3">

</xml_diff>